<commit_message>
feat(planilla): columna ROL por operador en plantilla de pago
- Plantilla nueva Planilla_Logistica_Eventos2.xlsx (ROL en H, resto +1 col hasta N, LUGAR K7->J7)
- planilla_excel.py: COL_ROL=8, COL_COORDINADOR=9, COL_CHAQ=10, COL_GORRA=11, COL_FIRMA=13, LAST_COL=14, CELL_LUGAR=J7; _fill_operators escribe role_name
- planilla_pdf.py: print_area ampliado a B:N
- tests: asserts de ROL en structure y endpoint tests + nuevo test_planilla_rol_column_and_layout
</commit_message>
<xml_diff>
--- a/backend/app/templates/Planilla_Logistica_Eventos.xlsx
+++ b/backend/app/templates/Planilla_Logistica_Eventos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Karen\Downloads\logistica\backend\app\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Karen\Downloads\logistica\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53668A79-A009-4147-8824-BC008629421A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{62735CBF-A638-4AF1-AAC6-B06A6383A951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,9 +16,10 @@
     <sheet name="Planilla" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Planilla!$B$2:$M$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Planilla!$B$2:$N$28</definedName>
   </definedNames>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>LOGISTICA DE EVENTOS</t>
   </si>
@@ -103,13 +104,16 @@
   </si>
   <si>
     <t>PLANILLA DE PAGO - SOPORTE CUENTA DE COBRO</t>
+  </si>
+  <si>
+    <t>ROL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,14 +146,6 @@
       <b/>
       <sz val="18"/>
       <color theme="2" tint="-0.249977111117893"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="16"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -332,7 +328,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -346,6 +342,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -355,6 +354,24 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -408,24 +425,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -787,7 +786,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:N36"/>
+  <dimension ref="B2:O36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="23.25" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
@@ -796,131 +795,137 @@
     <col min="4" max="4" width="40.140625" style="2" customWidth="1"/>
     <col min="5" max="5" width="31.42578125" style="2" customWidth="1"/>
     <col min="6" max="6" width="39.85546875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="39.5703125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="24" style="2" customWidth="1"/>
-    <col min="9" max="10" width="12" style="2" customWidth="1"/>
-    <col min="11" max="11" width="17.85546875" style="2" customWidth="1"/>
-    <col min="12" max="12" width="26.140625" style="2" customWidth="1"/>
-    <col min="13" max="13" width="12" style="2" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="2"/>
+    <col min="7" max="8" width="39.5703125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="24" style="2" customWidth="1"/>
+    <col min="10" max="11" width="12" style="2" customWidth="1"/>
+    <col min="12" max="12" width="24.7109375" style="2" customWidth="1"/>
+    <col min="13" max="13" width="45.7109375" style="2" customWidth="1"/>
+    <col min="14" max="14" width="32" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="21"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="7" t="s">
+    <row r="2" spans="2:15" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="28"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="8"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="7" t="s">
+      <c r="E2" s="9"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
       <c r="J2" s="9"/>
-      <c r="K2" s="28" t="s">
+      <c r="K2" s="10"/>
+      <c r="L2" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="L2" s="29"/>
-      <c r="M2" s="30"/>
-      <c r="N2" s="1"/>
-    </row>
-    <row r="3" spans="2:14" ht="53.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="23"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="7" t="s">
+      <c r="M2" s="12"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="1"/>
+    </row>
+    <row r="3" spans="2:15" ht="53.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="30"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="8"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="7" t="s">
+      <c r="E3" s="9"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
       <c r="J3" s="9"/>
-      <c r="K3" s="31"/>
-      <c r="L3" s="32"/>
-      <c r="M3" s="33"/>
-      <c r="N3" s="1"/>
-    </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B4" s="25"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
-      <c r="H4" s="26"/>
-      <c r="I4" s="26"/>
-      <c r="J4" s="26"/>
-      <c r="K4" s="26"/>
-      <c r="L4" s="26"/>
-      <c r="M4" s="27"/>
-      <c r="N4" s="1"/>
-    </row>
-    <row r="5" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="1"/>
+    </row>
+    <row r="4" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B4" s="32"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
+      <c r="I4" s="33"/>
+      <c r="J4" s="33"/>
+      <c r="K4" s="33"/>
+      <c r="L4" s="33"/>
+      <c r="M4" s="33"/>
+      <c r="N4" s="34"/>
+      <c r="O4" s="1"/>
+    </row>
+    <row r="5" spans="2:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="17"/>
       <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="3" t="s">
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="L5" s="19" t="s">
+      <c r="M5" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="M5" s="20"/>
-      <c r="N5" s="1"/>
-    </row>
-    <row r="6" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="11"/>
+      <c r="N5" s="27"/>
+      <c r="O5" s="1"/>
+    </row>
+    <row r="6" spans="2:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="18"/>
       <c r="C6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="13"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="16" t="s">
+      <c r="D6" s="20"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="I6" s="18"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="13" t="s">
+      <c r="J6" s="25"/>
+      <c r="K6" s="24"/>
+      <c r="L6" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="L6" s="14"/>
-      <c r="M6" s="15"/>
-      <c r="N6" s="1"/>
-    </row>
-    <row r="7" spans="2:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="12"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="1"/>
+    </row>
+    <row r="7" spans="2:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="19"/>
       <c r="C7" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="13"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="16" t="s">
+      <c r="D7" s="20"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="21"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="J7" s="17"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="14"/>
-      <c r="M7" s="15"/>
-    </row>
-    <row r="8" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K7" s="24"/>
+      <c r="L7" s="20"/>
+      <c r="M7" s="21"/>
+      <c r="N7" s="22"/>
+    </row>
+    <row r="8" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="4" t="s">
         <v>7</v>
       </c>
@@ -940,25 +945,28 @@
         <v>12</v>
       </c>
       <c r="H8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="J8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="K8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="L8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="L8" s="4" t="s">
+      <c r="M8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="M8" s="4" t="s">
+      <c r="N8" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="2:14" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:15" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="5">
         <v>1</v>
       </c>
@@ -973,8 +981,9 @@
       <c r="K9" s="5"/>
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
-    </row>
-    <row r="10" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N9" s="5"/>
+    </row>
+    <row r="10" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="5">
         <v>2</v>
       </c>
@@ -989,8 +998,9 @@
       <c r="K10" s="5"/>
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
-    </row>
-    <row r="11" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N10" s="5"/>
+    </row>
+    <row r="11" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="5">
         <v>3</v>
       </c>
@@ -1005,8 +1015,9 @@
       <c r="K11" s="5"/>
       <c r="L11" s="5"/>
       <c r="M11" s="5"/>
-    </row>
-    <row r="12" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N11" s="5"/>
+    </row>
+    <row r="12" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="5">
         <v>4</v>
       </c>
@@ -1021,8 +1032,9 @@
       <c r="K12" s="5"/>
       <c r="L12" s="5"/>
       <c r="M12" s="5"/>
-    </row>
-    <row r="13" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N12" s="5"/>
+    </row>
+    <row r="13" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="5">
         <v>5</v>
       </c>
@@ -1037,8 +1049,9 @@
       <c r="K13" s="5"/>
       <c r="L13" s="5"/>
       <c r="M13" s="5"/>
-    </row>
-    <row r="14" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N13" s="5"/>
+    </row>
+    <row r="14" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="5">
         <v>6</v>
       </c>
@@ -1053,8 +1066,9 @@
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
       <c r="M14" s="5"/>
-    </row>
-    <row r="15" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N14" s="5"/>
+    </row>
+    <row r="15" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="5">
         <v>7</v>
       </c>
@@ -1069,8 +1083,9 @@
       <c r="K15" s="5"/>
       <c r="L15" s="5"/>
       <c r="M15" s="5"/>
-    </row>
-    <row r="16" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N15" s="5"/>
+    </row>
+    <row r="16" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="5">
         <v>8</v>
       </c>
@@ -1085,8 +1100,9 @@
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
       <c r="M16" s="5"/>
-    </row>
-    <row r="17" spans="2:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N16" s="5"/>
+    </row>
+    <row r="17" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="5">
         <v>9</v>
       </c>
@@ -1101,8 +1117,9 @@
       <c r="K17" s="5"/>
       <c r="L17" s="5"/>
       <c r="M17" s="5"/>
-    </row>
-    <row r="18" spans="2:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N17" s="5"/>
+    </row>
+    <row r="18" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="5">
         <v>10</v>
       </c>
@@ -1117,8 +1134,9 @@
       <c r="K18" s="5"/>
       <c r="L18" s="5"/>
       <c r="M18" s="5"/>
-    </row>
-    <row r="19" spans="2:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N18" s="5"/>
+    </row>
+    <row r="19" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="5">
         <v>11</v>
       </c>
@@ -1133,8 +1151,9 @@
       <c r="K19" s="5"/>
       <c r="L19" s="5"/>
       <c r="M19" s="5"/>
-    </row>
-    <row r="20" spans="2:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N19" s="5"/>
+    </row>
+    <row r="20" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="5">
         <v>12</v>
       </c>
@@ -1149,8 +1168,9 @@
       <c r="K20" s="5"/>
       <c r="L20" s="5"/>
       <c r="M20" s="5"/>
-    </row>
-    <row r="21" spans="2:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N20" s="5"/>
+    </row>
+    <row r="21" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="5">
         <v>13</v>
       </c>
@@ -1165,8 +1185,9 @@
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
       <c r="M21" s="5"/>
-    </row>
-    <row r="22" spans="2:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N21" s="5"/>
+    </row>
+    <row r="22" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="5">
         <v>14</v>
       </c>
@@ -1181,8 +1202,9 @@
       <c r="K22" s="5"/>
       <c r="L22" s="5"/>
       <c r="M22" s="5"/>
-    </row>
-    <row r="23" spans="2:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N22" s="5"/>
+    </row>
+    <row r="23" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="5">
         <v>15</v>
       </c>
@@ -1197,8 +1219,9 @@
       <c r="K23" s="5"/>
       <c r="L23" s="5"/>
       <c r="M23" s="5"/>
-    </row>
-    <row r="24" spans="2:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N23" s="5"/>
+    </row>
+    <row r="24" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="5">
         <v>16</v>
       </c>
@@ -1213,8 +1236,9 @@
       <c r="K24" s="5"/>
       <c r="L24" s="5"/>
       <c r="M24" s="5"/>
-    </row>
-    <row r="25" spans="2:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N24" s="5"/>
+    </row>
+    <row r="25" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="5">
         <v>17</v>
       </c>
@@ -1229,8 +1253,9 @@
       <c r="K25" s="5"/>
       <c r="L25" s="5"/>
       <c r="M25" s="5"/>
-    </row>
-    <row r="26" spans="2:13" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N25" s="5"/>
+    </row>
+    <row r="26" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="5">
         <v>18</v>
       </c>
@@ -1245,8 +1270,9 @@
       <c r="K26" s="5"/>
       <c r="L26" s="5"/>
       <c r="M26" s="5"/>
-    </row>
-    <row r="27" spans="2:13" ht="39" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N26" s="5"/>
+    </row>
+    <row r="27" spans="2:14" ht="39" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="5">
         <v>19</v>
       </c>
@@ -1261,8 +1287,9 @@
       <c r="K27" s="5"/>
       <c r="L27" s="5"/>
       <c r="M27" s="5"/>
-    </row>
-    <row r="28" spans="2:13" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N27" s="5"/>
+    </row>
+    <row r="28" spans="2:14" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="5">
         <v>20</v>
       </c>
@@ -1277,11 +1304,12 @@
       <c r="K28" s="5"/>
       <c r="L28" s="5"/>
       <c r="M28" s="5"/>
-    </row>
-    <row r="29" spans="2:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="30" spans="2:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="31" spans="2:13" ht="24.95" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="34" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="N28" s="5"/>
+    </row>
+    <row r="29" spans="2:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="30" spans="2:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="31" spans="2:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="34" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B34" s="6"/>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
@@ -1294,8 +1322,9 @@
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
-    </row>
-    <row r="35" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="N34" s="1"/>
+    </row>
+    <row r="35" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
@@ -1308,8 +1337,9 @@
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
-    </row>
-    <row r="36" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="N35" s="1"/>
+    </row>
+    <row r="36" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
@@ -1322,27 +1352,28 @@
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
+      <c r="N36" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="D3:F3"/>
-    <mergeCell ref="G2:J2"/>
-    <mergeCell ref="G3:J3"/>
-    <mergeCell ref="K2:M3"/>
+    <mergeCell ref="G2:K2"/>
+    <mergeCell ref="G3:K3"/>
+    <mergeCell ref="L2:N3"/>
     <mergeCell ref="B5:B7"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="H6:J6"/>
-    <mergeCell ref="K7:M7"/>
-    <mergeCell ref="K6:M6"/>
-    <mergeCell ref="L5:M5"/>
-    <mergeCell ref="D5:J5"/>
+    <mergeCell ref="D7:I7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="I6:K6"/>
+    <mergeCell ref="L7:N7"/>
+    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="M5:N5"/>
+    <mergeCell ref="D5:K5"/>
     <mergeCell ref="D6:G6"/>
     <mergeCell ref="B2:C3"/>
-    <mergeCell ref="B4:M4"/>
+    <mergeCell ref="B4:N4"/>
     <mergeCell ref="D2:F2"/>
   </mergeCells>
-  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.98425196850393704" bottom="0.39370078740157483" header="0.51181102362204722" footer="0.39370078740157483"/>
   <pageSetup scale="42" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>

<commit_message>
chore(planilla): plantilla Excel con campos mas grandes
- Columna C mas ancha (44.9 -> 48.3) y columna K con ancho definido
- Alturas de fila ampliadas (filas 5-7: 27pt, filas 8-28: 57.75pt)
- Estructura intacta: mismos merges, headers y celdas de datos
  (verificado celda por celda); tests de nomina 4/4 OK
</commit_message>
<xml_diff>
--- a/backend/app/templates/Planilla_Logistica_Eventos.xlsx
+++ b/backend/app/templates/Planilla_Logistica_Eventos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Karen\Downloads\logistica\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{62735CBF-A638-4AF1-AAC6-B06A6383A951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B680B39B-1989-4F91-8E25-605AF00055E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,6 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">Planilla!$B$2:$N$28</definedName>
   </definedNames>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -113,7 +112,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -146,6 +145,20 @@
       <b/>
       <sz val="18"/>
       <color theme="2" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -328,7 +341,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -426,6 +439,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -791,13 +808,14 @@
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
     <col min="2" max="2" width="6" style="2" customWidth="1"/>
-    <col min="3" max="3" width="44.85546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="48.28515625" style="2" customWidth="1"/>
     <col min="4" max="4" width="40.140625" style="2" customWidth="1"/>
     <col min="5" max="5" width="31.42578125" style="2" customWidth="1"/>
     <col min="6" max="6" width="39.85546875" style="2" customWidth="1"/>
     <col min="7" max="8" width="39.5703125" style="2" customWidth="1"/>
     <col min="9" max="9" width="24" style="2" customWidth="1"/>
-    <col min="10" max="11" width="12" style="2" customWidth="1"/>
+    <col min="10" max="10" width="14" style="2" customWidth="1"/>
+    <col min="11" max="11" width="12" style="2" customWidth="1"/>
     <col min="12" max="12" width="24.7109375" style="2" customWidth="1"/>
     <col min="13" max="13" width="45.7109375" style="2" customWidth="1"/>
     <col min="14" max="14" width="32" style="2" customWidth="1"/>
@@ -862,9 +880,9 @@
       <c r="N4" s="34"/>
       <c r="O4" s="1"/>
     </row>
-    <row r="5" spans="2:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:15" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="17"/>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="36" t="s">
         <v>5</v>
       </c>
       <c r="D5" s="21"/>
@@ -884,7 +902,7 @@
       <c r="N5" s="27"/>
       <c r="O5" s="1"/>
     </row>
-    <row r="6" spans="2:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:15" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="18"/>
       <c r="C6" s="3" t="s">
         <v>1</v>
@@ -906,7 +924,7 @@
       <c r="N6" s="22"/>
       <c r="O6" s="1"/>
     </row>
-    <row r="7" spans="2:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:15" ht="27" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="19"/>
       <c r="C7" s="3" t="s">
         <v>3</v>
@@ -925,7 +943,7 @@
       <c r="M7" s="21"/>
       <c r="N7" s="22"/>
     </row>
-    <row r="8" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="4" t="s">
         <v>7</v>
       </c>
@@ -950,10 +968,10 @@
       <c r="I8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="J8" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="K8" s="35" t="s">
         <v>15</v>
       </c>
       <c r="L8" s="4" t="s">
@@ -966,7 +984,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="2:15" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="5">
         <v>1</v>
       </c>
@@ -983,7 +1001,7 @@
       <c r="M9" s="5"/>
       <c r="N9" s="5"/>
     </row>
-    <row r="10" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="5">
         <v>2</v>
       </c>
@@ -1000,7 +1018,7 @@
       <c r="M10" s="5"/>
       <c r="N10" s="5"/>
     </row>
-    <row r="11" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="5">
         <v>3</v>
       </c>
@@ -1017,7 +1035,7 @@
       <c r="M11" s="5"/>
       <c r="N11" s="5"/>
     </row>
-    <row r="12" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="5">
         <v>4</v>
       </c>
@@ -1034,7 +1052,7 @@
       <c r="M12" s="5"/>
       <c r="N12" s="5"/>
     </row>
-    <row r="13" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="5">
         <v>5</v>
       </c>
@@ -1051,7 +1069,7 @@
       <c r="M13" s="5"/>
       <c r="N13" s="5"/>
     </row>
-    <row r="14" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="5">
         <v>6</v>
       </c>
@@ -1068,7 +1086,7 @@
       <c r="M14" s="5"/>
       <c r="N14" s="5"/>
     </row>
-    <row r="15" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="5">
         <v>7</v>
       </c>
@@ -1085,7 +1103,7 @@
       <c r="M15" s="5"/>
       <c r="N15" s="5"/>
     </row>
-    <row r="16" spans="2:15" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="5">
         <v>8</v>
       </c>
@@ -1102,7 +1120,7 @@
       <c r="M16" s="5"/>
       <c r="N16" s="5"/>
     </row>
-    <row r="17" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:14" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="5">
         <v>9</v>
       </c>
@@ -1119,7 +1137,7 @@
       <c r="M17" s="5"/>
       <c r="N17" s="5"/>
     </row>
-    <row r="18" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:14" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="5">
         <v>10</v>
       </c>
@@ -1136,7 +1154,7 @@
       <c r="M18" s="5"/>
       <c r="N18" s="5"/>
     </row>
-    <row r="19" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:14" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="5">
         <v>11</v>
       </c>
@@ -1153,7 +1171,7 @@
       <c r="M19" s="5"/>
       <c r="N19" s="5"/>
     </row>
-    <row r="20" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:14" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="5">
         <v>12</v>
       </c>
@@ -1170,7 +1188,7 @@
       <c r="M20" s="5"/>
       <c r="N20" s="5"/>
     </row>
-    <row r="21" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:14" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="5">
         <v>13</v>
       </c>
@@ -1187,7 +1205,7 @@
       <c r="M21" s="5"/>
       <c r="N21" s="5"/>
     </row>
-    <row r="22" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:14" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="5">
         <v>14</v>
       </c>
@@ -1204,7 +1222,7 @@
       <c r="M22" s="5"/>
       <c r="N22" s="5"/>
     </row>
-    <row r="23" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:14" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="5">
         <v>15</v>
       </c>
@@ -1221,7 +1239,7 @@
       <c r="M23" s="5"/>
       <c r="N23" s="5"/>
     </row>
-    <row r="24" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:14" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="5">
         <v>16</v>
       </c>
@@ -1238,7 +1256,7 @@
       <c r="M24" s="5"/>
       <c r="N24" s="5"/>
     </row>
-    <row r="25" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:14" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="5">
         <v>17</v>
       </c>
@@ -1255,7 +1273,7 @@
       <c r="M25" s="5"/>
       <c r="N25" s="5"/>
     </row>
-    <row r="26" spans="2:14" ht="42" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:14" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="5">
         <v>18</v>
       </c>
@@ -1272,7 +1290,7 @@
       <c r="M26" s="5"/>
       <c r="N26" s="5"/>
     </row>
-    <row r="27" spans="2:14" ht="39" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:14" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="5">
         <v>19</v>
       </c>
@@ -1289,7 +1307,7 @@
       <c r="M27" s="5"/>
       <c r="N27" s="5"/>
     </row>
-    <row r="28" spans="2:14" ht="40.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:14" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="5">
         <v>20</v>
       </c>
@@ -1375,7 +1393,7 @@
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.98425196850393704" bottom="0.39370078740157483" header="0.51181102362204722" footer="0.39370078740157483"/>
-  <pageSetup scale="42" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="32" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualziación de la plantilla de planilla logística de eventos, corrección de las margenes
</commit_message>
<xml_diff>
--- a/backend/app/templates/Planilla_Logistica_Eventos.xlsx
+++ b/backend/app/templates/Planilla_Logistica_Eventos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Karen\Downloads\logistica\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Karen\Downloads\logistica\backend\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B680B39B-1989-4F91-8E25-605AF00055E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BE0B7FA-3698-4474-B66D-0CEC1184883F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilla" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Planilla!$B$2:$N$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Planilla!$A$1:$O$30</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <extLst>
@@ -358,6 +358,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -439,10 +443,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -823,125 +823,125 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:15" ht="47.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="28"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="8" t="s">
+      <c r="B2" s="30"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="9"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="8" t="s">
+      <c r="E2" s="11"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="11" t="s">
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="M2" s="12"/>
-      <c r="N2" s="13"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="15"/>
       <c r="O2" s="1"/>
     </row>
     <row r="3" spans="2:15" ht="53.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="30"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="8" t="s">
+      <c r="B3" s="32"/>
+      <c r="C3" s="33"/>
+      <c r="D3" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="9"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="8" t="s">
+      <c r="E3" s="11"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="15"/>
-      <c r="N3" s="16"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="17"/>
+      <c r="N3" s="18"/>
       <c r="O3" s="1"/>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B4" s="32"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="33"/>
-      <c r="G4" s="33"/>
-      <c r="H4" s="33"/>
-      <c r="I4" s="33"/>
-      <c r="J4" s="33"/>
-      <c r="K4" s="33"/>
-      <c r="L4" s="33"/>
-      <c r="M4" s="33"/>
-      <c r="N4" s="34"/>
+      <c r="B4" s="34"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="35"/>
+      <c r="K4" s="35"/>
+      <c r="L4" s="35"/>
+      <c r="M4" s="35"/>
+      <c r="N4" s="36"/>
       <c r="O4" s="1"/>
     </row>
     <row r="5" spans="2:15" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="17"/>
-      <c r="C5" s="36" t="s">
+      <c r="B5" s="19"/>
+      <c r="C5" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="21"/>
-      <c r="H5" s="21"/>
-      <c r="I5" s="21"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="22"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
+      <c r="I5" s="23"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="24"/>
       <c r="L5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="M5" s="26" t="s">
+      <c r="M5" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="N5" s="27"/>
+      <c r="N5" s="29"/>
       <c r="O5" s="1"/>
     </row>
     <row r="6" spans="2:15" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="18"/>
+      <c r="B6" s="20"/>
       <c r="C6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="20"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="24"/>
       <c r="H6" s="7"/>
-      <c r="I6" s="23" t="s">
+      <c r="I6" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="J6" s="25"/>
-      <c r="K6" s="24"/>
-      <c r="L6" s="20" t="s">
+      <c r="J6" s="27"/>
+      <c r="K6" s="26"/>
+      <c r="L6" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="M6" s="21"/>
-      <c r="N6" s="22"/>
+      <c r="M6" s="23"/>
+      <c r="N6" s="24"/>
       <c r="O6" s="1"/>
     </row>
     <row r="7" spans="2:15" ht="27" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="19"/>
+      <c r="B7" s="21"/>
       <c r="C7" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="20"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="21"/>
-      <c r="I7" s="22"/>
-      <c r="J7" s="23" t="s">
+      <c r="D7" s="22"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="K7" s="24"/>
-      <c r="L7" s="20"/>
-      <c r="M7" s="21"/>
-      <c r="N7" s="22"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="24"/>
     </row>
     <row r="8" spans="2:15" ht="57.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="4" t="s">
@@ -968,10 +968,10 @@
       <c r="I8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="J8" s="35" t="s">
+      <c r="J8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="35" t="s">
+      <c r="K8" s="8" t="s">
         <v>15</v>
       </c>
       <c r="L8" s="4" t="s">
@@ -1392,8 +1392,8 @@
     <mergeCell ref="D2:F2"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.98425196850393704" bottom="0.39370078740157483" header="0.51181102362204722" footer="0.39370078740157483"/>
-  <pageSetup scale="32" orientation="landscape" r:id="rId1"/>
+  <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="1.9685039370078741" bottom="0.39370078740157483" header="0.98425196850393704" footer="0.39370078740157483"/>
+  <pageSetup scale="30" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>